<commit_message>
Vector Store practice with FAISS
</commit_message>
<xml_diff>
--- a/sample_files/office/quarterly_sales.xlsx
+++ b/sample_files/office/quarterly_sales.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,38 +468,6 @@
       </c>
       <c r="D3" t="n">
         <v>50000</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Mar</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>135000</v>
-      </c>
-      <c r="C4" t="n">
-        <v>88000</v>
-      </c>
-      <c r="D4" t="n">
-        <v>47000</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Apr</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>150000</v>
-      </c>
-      <c r="C5" t="n">
-        <v>93000</v>
-      </c>
-      <c r="D5" t="n">
-        <v>57000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>